<commit_message>
GBDS MARCH FILES 2026 | fliqlo@GBDS
</commit_message>
<xml_diff>
--- a/GBDS MARCH FILES 2026/CSR MONTH OF MARCH 2026.xlsx
+++ b/GBDS MARCH FILES 2026/CSR MONTH OF MARCH 2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS APRIL FILES 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS MARCH FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A9BDC8-2079-45FC-B2B2-6651F0B10B18}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44EBA45-E627-4050-8A06-3EC7000D38A7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="28" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | APRIL" sheetId="902" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2471" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2489" uniqueCount="89">
   <si>
     <t>CHECKER STOCK REPORT</t>
   </si>
@@ -323,6 +323,42 @@
   </si>
   <si>
     <t>DATE ___________03/09/2026___________</t>
+  </si>
+  <si>
+    <t>6/5b</t>
+  </si>
+  <si>
+    <t>6/23b</t>
+  </si>
+  <si>
+    <t>13/4b</t>
+  </si>
+  <si>
+    <t>2/12b</t>
+  </si>
+  <si>
+    <t>12b</t>
+  </si>
+  <si>
+    <t>9/3b</t>
+  </si>
+  <si>
+    <t>10/12b</t>
+  </si>
+  <si>
+    <t>1/12b</t>
+  </si>
+  <si>
+    <t>3/4b</t>
+  </si>
+  <si>
+    <t>12/8b</t>
+  </si>
+  <si>
+    <t>5/20b</t>
+  </si>
+  <si>
+    <t>18/4b</t>
   </si>
 </sst>
 </file>
@@ -1202,15 +1238,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1220,22 +1247,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3062,40 +3098,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -3103,7 +3139,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -3335,12 +3371,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -4667,40 +4703,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -4708,7 +4744,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -4940,12 +4976,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -4981,17 +5017,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -6290,40 +6326,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -6331,7 +6367,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -6563,12 +6599,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -6604,17 +6640,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7913,40 +7949,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -7954,7 +7990,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -8186,12 +8222,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -8227,17 +8263,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9534,40 +9570,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -9575,7 +9611,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -9807,12 +9843,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -11139,40 +11175,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -11180,7 +11216,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -11412,12 +11448,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -11453,17 +11489,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -12762,40 +12798,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -12803,7 +12839,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -13035,12 +13071,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -13076,17 +13112,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -14385,40 +14421,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -14426,7 +14462,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -14658,12 +14694,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -14699,17 +14735,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -16006,40 +16042,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -16047,7 +16083,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -16279,12 +16315,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -17611,40 +17647,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -17652,7 +17688,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -17884,12 +17920,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -17925,17 +17961,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -19232,40 +19268,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -19273,7 +19309,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -19505,12 +19541,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -20837,40 +20873,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -20878,7 +20914,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -21110,12 +21146,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -21151,17 +21187,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -22460,40 +22496,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -22501,7 +22537,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -22733,12 +22769,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -22774,17 +22810,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -24081,40 +24117,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -24122,7 +24158,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -24354,12 +24390,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -25686,40 +25722,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -25727,7 +25763,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -25959,12 +25995,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -26000,17 +26036,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -27309,40 +27345,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -27350,7 +27386,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -27582,12 +27618,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -27623,17 +27659,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -28932,40 +28968,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -28973,7 +29009,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -29205,12 +29241,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -29246,17 +29282,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -30553,40 +30589,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -30594,7 +30630,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -30826,12 +30862,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -32158,40 +32194,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -32199,7 +32235,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -32431,12 +32467,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -32472,17 +32508,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -33781,40 +33817,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -33822,7 +33858,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -34054,12 +34090,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -34095,17 +34131,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -35404,40 +35440,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -35445,7 +35481,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -35677,12 +35713,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -35718,17 +35754,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -36125,12 +36161,20 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="13">
+        <v>1</v>
+      </c>
+      <c r="D8" s="14">
+        <v>1</v>
+      </c>
       <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
+      <c r="F8" s="14">
+        <v>1</v>
+      </c>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -36140,12 +36184,18 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
+      <c r="R8" s="14">
+        <v>2</v>
+      </c>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>2</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>3</v>
+      </c>
       <c r="X8" s="60"/>
       <c r="Y8" s="15"/>
     </row>
@@ -36313,12 +36363,20 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
+      <c r="C15" s="22">
+        <v>0</v>
+      </c>
+      <c r="D15" s="23">
+        <v>0</v>
+      </c>
       <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
+      <c r="F15" s="23">
+        <v>0</v>
+      </c>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>78</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -36328,12 +36386,18 @@
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
+      <c r="R15" s="23">
+        <v>2</v>
+      </c>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>2</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>1</v>
+      </c>
       <c r="X15" s="62"/>
       <c r="Y15" s="24"/>
     </row>
@@ -36341,12 +36405,20 @@
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
+      <c r="C16" s="58">
+        <v>1</v>
+      </c>
+      <c r="D16" s="59">
+        <v>1</v>
+      </c>
       <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
+      <c r="F16" s="27">
+        <v>1</v>
+      </c>
       <c r="G16" s="28"/>
-      <c r="H16" s="65"/>
+      <c r="H16" s="65" t="s">
+        <v>77</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="57"/>
@@ -36356,12 +36428,18 @@
       <c r="O16" s="28"/>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
+      <c r="R16" s="28">
+        <v>0</v>
+      </c>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>0</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="57"/>
+      <c r="W16" s="57">
+        <v>2</v>
+      </c>
       <c r="X16" s="63"/>
       <c r="Y16" s="29"/>
     </row>
@@ -36765,17 +36843,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>19</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>1</v>
+      </c>
+      <c r="L24" s="14">
+        <v>12</v>
+      </c>
+      <c r="M24" s="14">
+        <v>325</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14">
+        <v>5</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -36951,17 +37041,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23" t="s">
+        <v>81</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>1</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>0</v>
+      </c>
+      <c r="L31" s="23">
+        <v>0</v>
+      </c>
+      <c r="M31" s="23">
+        <v>17</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23">
+        <v>5</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -36979,17 +37081,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>2</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>18</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>1</v>
+      </c>
+      <c r="L32" s="28">
+        <v>12</v>
+      </c>
+      <c r="M32" s="28">
+        <v>308</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -37027,40 +37141,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -37068,7 +37182,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -37127,21 +37241,49 @@
       <c r="B36" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="47"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="43"/>
-      <c r="K36" s="43"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
+      <c r="C36" s="47">
+        <v>1</v>
+      </c>
+      <c r="D36" s="42">
+        <v>1</v>
+      </c>
+      <c r="E36" s="43">
+        <v>20</v>
+      </c>
+      <c r="F36" s="43">
+        <v>240</v>
+      </c>
+      <c r="G36" s="43">
+        <v>1</v>
+      </c>
+      <c r="H36" s="43">
+        <v>1</v>
+      </c>
+      <c r="I36" s="43">
+        <v>22</v>
+      </c>
+      <c r="J36" s="43">
+        <v>1</v>
+      </c>
+      <c r="K36" s="43">
+        <v>7</v>
+      </c>
+      <c r="L36" s="43">
+        <v>3</v>
+      </c>
+      <c r="M36" s="43">
+        <v>2</v>
+      </c>
+      <c r="N36" s="43">
+        <v>11</v>
+      </c>
+      <c r="O36" s="43">
+        <v>7</v>
+      </c>
       <c r="P36" s="43"/>
-      <c r="Q36" s="44"/>
+      <c r="Q36" s="44">
+        <v>3</v>
+      </c>
       <c r="R36" s="76"/>
       <c r="S36" s="66"/>
       <c r="T36" s="66"/>
@@ -37285,27 +37427,55 @@
       <c r="B42" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="47"/>
-      <c r="D42" s="42"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
-      <c r="J42" s="43"/>
-      <c r="K42" s="43"/>
-      <c r="L42" s="43"/>
-      <c r="M42" s="43"/>
-      <c r="N42" s="43"/>
-      <c r="O42" s="43"/>
+      <c r="C42" s="47">
+        <v>1</v>
+      </c>
+      <c r="D42" s="42">
+        <v>1</v>
+      </c>
+      <c r="E42" s="43">
+        <v>20</v>
+      </c>
+      <c r="F42" s="43">
+        <v>240</v>
+      </c>
+      <c r="G42" s="43">
+        <v>1</v>
+      </c>
+      <c r="H42" s="43">
+        <v>1</v>
+      </c>
+      <c r="I42" s="43">
+        <v>22</v>
+      </c>
+      <c r="J42" s="43">
+        <v>1</v>
+      </c>
+      <c r="K42" s="43">
+        <v>7</v>
+      </c>
+      <c r="L42" s="43">
+        <v>3</v>
+      </c>
+      <c r="M42" s="43">
+        <v>2</v>
+      </c>
+      <c r="N42" s="43">
+        <v>11</v>
+      </c>
+      <c r="O42" s="43">
+        <v>7</v>
+      </c>
       <c r="P42" s="43"/>
-      <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="Q42" s="44">
+        <v>3</v>
+      </c>
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -37341,17 +37511,23 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95">
+        <f>1+1+1+6+2+2+18+1+12+308</f>
+        <v>352</v>
+      </c>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -37379,7 +37555,9 @@
   <cols>
     <col min="1" max="1" width="1.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="2" customWidth="1"/>
-    <col min="3" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="3" max="5" width="5.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="5.7109375" style="2" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="5.7109375" style="2" customWidth="1"/>
@@ -37748,12 +37926,18 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13" t="s">
+        <v>80</v>
+      </c>
       <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
+      <c r="E8" s="14">
+        <v>2</v>
+      </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>82</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -37763,14 +37947,20 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
+      <c r="R8" s="14">
+        <v>1</v>
+      </c>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>2</v>
+      </c>
       <c r="X8" s="60"/>
-      <c r="Y8" s="15"/>
+      <c r="Y8" s="15">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -37936,12 +38126,18 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
+      <c r="E15" s="23">
+        <v>0</v>
+      </c>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23">
+        <v>0</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -37951,25 +38147,37 @@
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
+      <c r="R15" s="23">
+        <v>1</v>
+      </c>
       <c r="S15" s="23"/>
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>2</v>
+      </c>
       <c r="X15" s="62"/>
-      <c r="Y15" s="24"/>
+      <c r="Y15" s="24">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="58"/>
+      <c r="C16" s="58">
+        <v>0</v>
+      </c>
       <c r="D16" s="59"/>
-      <c r="E16" s="27"/>
+      <c r="E16" s="27">
+        <v>2</v>
+      </c>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="65"/>
+      <c r="H16" s="65" t="s">
+        <v>82</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="57"/>
@@ -37979,14 +38187,20 @@
       <c r="O16" s="28"/>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
+      <c r="R16" s="28">
+        <v>0</v>
+      </c>
       <c r="S16" s="28"/>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="57"/>
+      <c r="W16" s="57">
+        <v>0</v>
+      </c>
       <c r="X16" s="63"/>
-      <c r="Y16" s="29"/>
+      <c r="Y16" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -38385,20 +38599,34 @@
       <c r="B24" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="13"/>
+      <c r="C24" s="13">
+        <v>1</v>
+      </c>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>40</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="L24" s="14">
+        <v>10</v>
+      </c>
+      <c r="M24" s="14">
+        <v>391</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -38571,20 +38799,34 @@
       <c r="B31" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="22"/>
+      <c r="C31" s="22">
+        <v>0</v>
+      </c>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>0</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>0</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>1</v>
+      </c>
+      <c r="L31" s="23">
+        <v>9</v>
+      </c>
+      <c r="M31" s="23">
+        <v>40</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>85</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -38599,20 +38841,34 @@
       <c r="B32" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C32" s="26"/>
+      <c r="C32" s="26">
+        <v>1</v>
+      </c>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27" t="s">
+        <v>83</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>40</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="L32" s="28">
+        <v>1</v>
+      </c>
+      <c r="M32" s="28">
+        <v>351</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -38650,40 +38906,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -38691,7 +38947,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -38750,21 +39006,45 @@
       <c r="B36" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="47"/>
+      <c r="C36" s="47">
+        <v>9</v>
+      </c>
       <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
+      <c r="E36" s="43">
+        <v>10</v>
+      </c>
+      <c r="F36" s="43">
+        <v>465</v>
+      </c>
+      <c r="G36" s="43">
+        <v>10</v>
+      </c>
+      <c r="H36" s="43">
+        <v>5</v>
+      </c>
+      <c r="I36" s="43">
+        <v>1</v>
+      </c>
       <c r="J36" s="43"/>
-      <c r="K36" s="43"/>
+      <c r="K36" s="43">
+        <v>2</v>
+      </c>
       <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="43"/>
-      <c r="Q36" s="44"/>
+      <c r="M36" s="43">
+        <v>1</v>
+      </c>
+      <c r="N36" s="43">
+        <v>36</v>
+      </c>
+      <c r="O36" s="43">
+        <v>6</v>
+      </c>
+      <c r="P36" s="43">
+        <v>22</v>
+      </c>
+      <c r="Q36" s="44">
+        <v>5</v>
+      </c>
       <c r="R36" s="76"/>
       <c r="S36" s="66"/>
       <c r="T36" s="66"/>
@@ -38908,27 +39188,51 @@
       <c r="B42" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="47"/>
+      <c r="C42" s="47">
+        <v>9</v>
+      </c>
       <c r="D42" s="42"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
+      <c r="E42" s="43">
+        <v>10</v>
+      </c>
+      <c r="F42" s="43">
+        <v>465</v>
+      </c>
+      <c r="G42" s="43">
+        <v>10</v>
+      </c>
+      <c r="H42" s="43">
+        <v>5</v>
+      </c>
+      <c r="I42" s="43">
+        <v>1</v>
+      </c>
       <c r="J42" s="43"/>
-      <c r="K42" s="43"/>
+      <c r="K42" s="43">
+        <v>2</v>
+      </c>
       <c r="L42" s="43"/>
-      <c r="M42" s="43"/>
-      <c r="N42" s="43"/>
-      <c r="O42" s="43"/>
-      <c r="P42" s="43"/>
-      <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="M42" s="43">
+        <v>1</v>
+      </c>
+      <c r="N42" s="43">
+        <v>36</v>
+      </c>
+      <c r="O42" s="43">
+        <v>6</v>
+      </c>
+      <c r="P42" s="43">
+        <v>22</v>
+      </c>
+      <c r="Q42" s="44">
+        <v>5</v>
+      </c>
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -38964,17 +39268,23 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95">
+        <f>2+9+1+10+40+1+351</f>
+        <v>414</v>
+      </c>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95">
+        <f>3+12</f>
+        <v>15</v>
+      </c>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -39371,12 +39681,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13">
+        <v>2</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>88</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -39386,14 +39700,20 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
+      <c r="R8" s="14">
+        <v>2</v>
+      </c>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>3</v>
+      </c>
       <c r="X8" s="60"/>
-      <c r="Y8" s="15"/>
+      <c r="Y8" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -39559,12 +39879,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22">
+        <v>2</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>87</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -39574,25 +39898,35 @@
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
+      <c r="R15" s="23">
+        <v>2</v>
+      </c>
       <c r="S15" s="23"/>
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>1</v>
+      </c>
       <c r="X15" s="62"/>
-      <c r="Y15" s="24"/>
+      <c r="Y15" s="24">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="58"/>
+      <c r="C16" s="58">
+        <v>0</v>
+      </c>
       <c r="D16" s="59"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="65"/>
+      <c r="H16" s="65" t="s">
+        <v>86</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="57"/>
@@ -39602,14 +39936,20 @@
       <c r="O16" s="28"/>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
+      <c r="R16" s="28">
+        <v>0</v>
+      </c>
       <c r="S16" s="28"/>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="57"/>
+      <c r="W16" s="57">
+        <v>2</v>
+      </c>
       <c r="X16" s="63"/>
-      <c r="Y16" s="29"/>
+      <c r="Y16" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -40011,23 +40351,37 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>3</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>111</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>2</v>
+      </c>
+      <c r="L24" s="14">
+        <v>15</v>
+      </c>
+      <c r="M24" s="14">
+        <v>421</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14">
+        <v>10</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
       <c r="T24" s="14"/>
       <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
+      <c r="V24" s="14">
+        <v>1</v>
+      </c>
       <c r="W24" s="14"/>
       <c r="X24" s="14"/>
       <c r="Y24" s="15"/>
@@ -40197,23 +40551,37 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>2</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>54</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>2</v>
+      </c>
+      <c r="L31" s="23">
+        <v>6</v>
+      </c>
+      <c r="M31" s="23">
+        <v>155</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23">
+        <v>10</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
       <c r="T31" s="23"/>
       <c r="U31" s="23"/>
-      <c r="V31" s="23"/>
+      <c r="V31" s="23">
+        <v>0</v>
+      </c>
       <c r="W31" s="23"/>
       <c r="X31" s="62"/>
       <c r="Y31" s="24"/>
@@ -40225,23 +40593,37 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>1</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>57</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>9</v>
+      </c>
+      <c r="M32" s="28">
+        <v>266</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
       <c r="T32" s="28"/>
       <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
+      <c r="V32" s="28">
+        <v>1</v>
+      </c>
       <c r="W32" s="28"/>
       <c r="X32" s="64"/>
       <c r="Y32" s="29"/>
@@ -40273,40 +40655,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -40314,7 +40696,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -40374,20 +40756,42 @@
         <v>52</v>
       </c>
       <c r="C36" s="47"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
+      <c r="D36" s="42">
+        <v>1</v>
+      </c>
+      <c r="E36" s="43">
+        <v>12</v>
+      </c>
+      <c r="F36" s="43">
+        <v>284</v>
+      </c>
+      <c r="G36" s="43">
+        <v>17</v>
+      </c>
       <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="43"/>
-      <c r="K36" s="43"/>
-      <c r="L36" s="43"/>
+      <c r="I36" s="43">
+        <v>16</v>
+      </c>
+      <c r="J36" s="43">
+        <v>1</v>
+      </c>
+      <c r="K36" s="43">
+        <v>10</v>
+      </c>
+      <c r="L36" s="43">
+        <v>2</v>
+      </c>
       <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
+      <c r="N36" s="43">
+        <v>10</v>
+      </c>
+      <c r="O36" s="43">
+        <v>12</v>
+      </c>
       <c r="P36" s="43"/>
-      <c r="Q36" s="44"/>
+      <c r="Q36" s="44">
+        <v>1</v>
+      </c>
       <c r="R36" s="76"/>
       <c r="S36" s="66"/>
       <c r="T36" s="66"/>
@@ -40532,26 +40936,48 @@
         <v>53</v>
       </c>
       <c r="C42" s="47"/>
-      <c r="D42" s="42"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="43"/>
+      <c r="D42" s="42">
+        <v>1</v>
+      </c>
+      <c r="E42" s="43">
+        <v>12</v>
+      </c>
+      <c r="F42" s="43">
+        <v>284</v>
+      </c>
+      <c r="G42" s="43">
+        <v>17</v>
+      </c>
       <c r="H42" s="43"/>
-      <c r="I42" s="43"/>
-      <c r="J42" s="43"/>
-      <c r="K42" s="43"/>
-      <c r="L42" s="43"/>
+      <c r="I42" s="43">
+        <v>16</v>
+      </c>
+      <c r="J42" s="43">
+        <v>1</v>
+      </c>
+      <c r="K42" s="43">
+        <v>10</v>
+      </c>
+      <c r="L42" s="43">
+        <v>2</v>
+      </c>
       <c r="M42" s="43"/>
-      <c r="N42" s="43"/>
-      <c r="O42" s="43"/>
+      <c r="N42" s="43">
+        <v>10</v>
+      </c>
+      <c r="O42" s="43">
+        <v>12</v>
+      </c>
       <c r="P42" s="43"/>
-      <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="Q42" s="44">
+        <v>1</v>
+      </c>
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -40587,17 +41013,23 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95">
+        <f>12+2+1+57+9+266+1</f>
+        <v>348</v>
+      </c>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -41894,40 +42326,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -41935,7 +42367,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -42167,12 +42599,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -43499,40 +43931,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -43540,7 +43972,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -43772,12 +44204,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -43813,17 +44245,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -45122,40 +45554,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -45163,7 +45595,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -45395,12 +45827,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -45436,17 +45868,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -46745,40 +47177,40 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="84" t="s">
+      <c r="D34" s="91"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="84" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="85"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="84" t="s">
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="85"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="93" t="s">
+      <c r="M34" s="91"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
-      <c r="R34" s="87" t="s">
+      <c r="P34" s="94"/>
+      <c r="Q34" s="94"/>
+      <c r="R34" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="88"/>
-      <c r="T34" s="88"/>
-      <c r="U34" s="89"/>
+      <c r="S34" s="85"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="86"/>
       <c r="V34" s="70"/>
       <c r="W34" s="67"/>
       <c r="X34" s="67"/>
@@ -46786,7 +47218,7 @@
       <c r="Z34" s="80"/>
     </row>
     <row r="35" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="91"/>
+      <c r="B35" s="90"/>
       <c r="C35" s="51" t="s">
         <v>49</v>
       </c>
@@ -47018,12 +47450,12 @@
       <c r="O42" s="43"/>
       <c r="P42" s="43"/>
       <c r="Q42" s="44"/>
-      <c r="R42" s="94" t="s">
+      <c r="R42" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="95"/>
-      <c r="T42" s="95"/>
-      <c r="U42" s="95"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
       <c r="V42" s="67"/>
       <c r="W42" s="67"/>
       <c r="X42" s="67"/>
@@ -47059,17 +47491,17 @@
       <c r="B44" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
-      <c r="D44" s="92"/>
-      <c r="E44" s="92"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="95"/>
     </row>
     <row r="45" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B45" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="92"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>